<commit_message>
Primer commit del Sistema PQR
</commit_message>
<xml_diff>
--- a/BaseDatos_PQR.xlsx
+++ b/BaseDatos_PQR.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="PQR" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Historial" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Investigaciones" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Adjuntos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PQR" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historial" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investigaciones" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adjuntos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:N39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12"/>
   <cols>
     <col width="14.140625" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -2279,6 +2279,167 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>PQR-2026-0038</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Reclamo</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Recibido</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Cambio de producto</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>[{"producto": "Z", "ref": "Z", "lote": "Z", "fechaEmp": "", "cant": "", "unidad": "Kilogramos", "tipoDoc": "Remisión", "numDoc": "ZZ"}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>PQR-2026-0039</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>12:18</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Sugerencia</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Yyyy</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Hhhh</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Hhhhjjjjjjjj</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Njjjjjj</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Recibido</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>PQR-2026-0040</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>12:26</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Queja</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Jjjj</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Recibido</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2290,7 +2451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3440,6 +3601,102 @@
         </is>
       </c>
       <c r="F36" t="inlineStr">
+        <is>
+          <t>PQR registrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>PQR-2026-0038</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Recibido</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>11:35:47</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>PQR registrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>PQR-2026-0039</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Recibido</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>12:19:12</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>PQR registrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>PQR-2026-0040</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Recibido</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>12:26:48</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
         <is>
           <t>PQR registrado</t>
         </is>
@@ -3874,7 +4131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4074,6 +4331,43 @@
         </is>
       </c>
       <c r="G6" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PQR-2026-0038</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Fotografía</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Captura_de_pantalla_2026-07-27_135034.png</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>📎 Abrir evidencia</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>11:35:47</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>Cliente</t>
         </is>
@@ -4085,6 +4379,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Corregir Base de datos para leer del Excel y reorganizar menú de perfiles
- Base de datos ahora usa la misma fuente que el Dashboard (hoja PQR del Excel) vía GET /api/pqr/todos, en lugar del localStorage del navegador

- Nueva función listar_pqrs() en excel_db.py; renderDB(), modales de estado y detalle sincronizados

- Sección Administración movida al menú del usuario, visible solo en Perfil Administrador
</commit_message>
<xml_diff>
--- a/BaseDatos_PQR.xlsx
+++ b/BaseDatos_PQR.xlsx
@@ -2136,7 +2136,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Recibido</t>
+          <t>En investigación</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2451,7 +2451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3699,6 +3699,70 @@
       <c r="F39" t="inlineStr">
         <is>
           <t>PQR registrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>PQR-2026-0035</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>En investigación</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>08:15:21</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Seguimiento actualizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>PQR-2026-0035</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>En investigación</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>08:15:22</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Seguimiento actualizado</t>
         </is>
       </c>
     </row>
@@ -3713,7 +3777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4117,6 +4181,38 @@
       <c r="K7" t="inlineStr">
         <is>
           <t>qqq</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PQR-2026-0035</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>5 ¿Por qué?</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Materias primas</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Reposición</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar contraseña administrador PQR
</commit_message>
<xml_diff>
--- a/BaseDatos_PQR.xlsx
+++ b/BaseDatos_PQR.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PQR" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historial" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investigaciones" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adjuntos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Usuarios" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="PQR" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Historial" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Investigaciones" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Adjuntos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Usuarios" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB9"/>
+  <dimension ref="A1:AB12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1339,6 +1339,411 @@
       <c r="AA9" t="inlineStr">
         <is>
           <t>Visita comercial</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PQR-2026-0009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>16:50</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Petición</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ELIAN S.A.S</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>10431226999</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>ELIAN BENITEZ</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>30172297700</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>elianbenitez56@gmail.com</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Recibido</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Cambio de producto</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>[{"linea": "INAPEL", "referencia_siesa": "M-421111", "detalle_presentacion": "RAYADO", "producto": "BLOCK FAMA ESCOLAR C/R CARTA 50HX70 UND", "unidad": "U", "lote": "102124", "fechaEmp": "2026-05-10", "cant": "200", "numDoc": "2055", "tipoDoc": "Factura de venta"}]</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>INAPEL</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>ELIAN</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>INAPEL</t>
+        </is>
+      </c>
+      <c r="R10" t="n">
+        <v>16</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>1043122544</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>elianbenitez56@gmail.com</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>3017229770</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>VENDEDOR</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>INAPEL</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>soledad</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Atlantico</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PQR-2026-0010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>17:11</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Reclamo</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>QQQQQQQQ</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>QQQQQQ</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>QQQQQQ</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>elianbeitez56@gmail.com</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Recibido</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Nota crédito</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>[{"linea": "INAPEL", "referencia_siesa": "M-421111", "detalle_presentacion": "RAYADO", "producto": "BLOCK FAMA ESCOLAR C/R CARTA 50HX70 UND", "unidad": "U", "lote": "", "fechaEmp": "", "cant": "", "numDoc": "", "tipoDoc": "Factura de venta"}]</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>INAPEL</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>ELIAN</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>INAPEL</t>
+        </is>
+      </c>
+      <c r="R11" t="n">
+        <v>16</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>1043122544</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>elianbenitez56@gmail.com</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>3017229770</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>VENDEDOR</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>INAPEL</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>QQQQ</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>Correo electrónico</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PQR-2026-0011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>17:21</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Queja</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>QQQQQQ</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>QQQQ</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>QQQQQQ</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>QQQQQ</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>proyectoautomatizacion27@gmail.com</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Recibido</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>qq</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Nota crédito</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>[{"linea": "INAPEL", "referencia_siesa": "M-421111", "detalle_presentacion": "CUADROS", "producto": "BLOCK FAMA ESCOLAR CUADROS CARTA 50HX70 UND", "unidad": "U", "lote": "", "fechaEmp": "", "cant": "", "numDoc": "", "tipoDoc": "Factura de venta"}]</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>INAPEL</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>ELIAN</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>INAPEL</t>
+        </is>
+      </c>
+      <c r="R12" t="n">
+        <v>16</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>1043122544</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>elianbenitez56@gmail.com</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>3017229770</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>VENDEDOR</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>INAPEL</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>QQ</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1801,6 +2206,102 @@
       <c r="F14" t="inlineStr">
         <is>
           <t>Seguimiento actualizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PQR-2026-0009</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Recibido</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>16:56:54</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>PQR registrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PQR-2026-0010</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Recibido</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>17:13:13</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>PQR registrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PQR-2026-0011</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Recibido</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>17:23:49</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>PQR registrado</t>
         </is>
       </c>
     </row>
@@ -1996,7 +2497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2147,6 +2648,80 @@
         </is>
       </c>
       <c r="G4" t="inlineStr">
+        <is>
+          <t>ELIAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PQR-2026-0009</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Fotografía</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Captura_de_pantalla_2026-09-02_165011.png</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>📎 Abrir evidencia</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>16:56:57</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>ELIAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PQR-2026-0010</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Captura_de_pantalla_2026-09-02_154423.png</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>📎 Abrir evidencia</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>17:13:15</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>ELIAN</t>
         </is>
@@ -2157,6 +2732,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2168,7 +2745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3003,7 +3580,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>scrypt:32768:8:1$IIUFsh66bmF4hNsW$384c1632a8f81e9fd53cf875cf11ea6a5b8ef129e3f2551f3c3467a05173715a09a95f6547373b17ef6a114b06aabee206a8c1a78898d2d34a6acb6f8d76b742</t>
+          <t>scrypt:32768:8:1$ry5XnIJw0F7JV4t3$11ff562697cccb8a86119be0f92487ea269077047967d89071e916a4b380bfc3589d5c5f821655c63b8e247b6f7bbef7c7be105039344d171d6f6f1db0b0bb87</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -3036,12 +3613,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1043122544</t>
+          <t>1043122699</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>scrypt:32768:8:1$pXpgxZWwrFAYFgEj$7280ca2446cb02accb4306e3866a83d202df973f702bf66a5cc9d28c92ebe1ad8731c7ff5131e5192012f4675e05a3e7eb0957e58fdf2460cb846b3f485d4623</t>
+          <t>scrypt:32768:8:1$JgAHa62TkqJkkRR2$4d7a46a08551804c1954fa7eeaf3af1b813ff95719529db6fb221bfdb61bbc870d1c71a7b3c95a651c48d5173fa1c000af72e91b939033ca33a77d746ac180e3</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -3312,6 +3889,49 @@
       <c r="L20" t="inlineStr">
         <is>
           <t>3215560240</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>23</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Pedro Luis Estrada Arias</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>pedro.estrada</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$lmfMgVav7Ly2ihME$1c7c7fe166827fc49375db41fb026b40bc290653670bc63078aae4b42db9f8296a3576e5154eb20ab63fe1329ac8ba497ab65a8cf2c5dc4990fa64a3a0ef1a1d</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LIDER_CALIDAD</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>INAPEL</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>INAPEL</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-09-02 16:42:37</t>
         </is>
       </c>
     </row>

</xml_diff>